<commit_message>
Changes on the project folders
</commit_message>
<xml_diff>
--- a/util/Validation/ToolValidation/longParamaterValidationForTool.xlsx
+++ b/util/Validation/ToolValidation/longParamaterValidationForTool.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x15 xr xr6 xr10">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10111"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/neda/Desktop/workspace/BadSmells/util/Validation/ToolValidation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{240EF6FA-D457-6D4A-BE16-B6B6DAF5398F}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B48ADD28-A6CE-6745-B3EF-44E80319CDC5}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="500" yWindow="460" windowWidth="25040" windowHeight="13760" activeTab="1"/>
+    <workbookView xWindow="500" yWindow="460" windowWidth="25040" windowHeight="13760" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="longParamaterValidationForTool" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet2" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">longParamaterValidationForTool!$A$1:$E$2133</definedName>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4768" uniqueCount="2159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4785" uniqueCount="2174">
   <si>
     <t>Method Name</t>
   </si>
@@ -6513,12 +6514,57 @@
   </si>
   <si>
     <t>nep_metadata</t>
+  </si>
+  <si>
+    <t>FN</t>
+  </si>
+  <si>
+    <t>TP</t>
+  </si>
+  <si>
+    <t>FP</t>
+  </si>
+  <si>
+    <t>Tool:</t>
+  </si>
+  <si>
+    <t>: Manuel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">recall = </t>
+  </si>
+  <si>
+    <t>TP/(TP + FP)</t>
+  </si>
+  <si>
+    <t>&gt;&gt;&gt;&gt;</t>
+  </si>
+  <si>
+    <t>204/(204+37)=0.846</t>
+  </si>
+  <si>
+    <t xml:space="preserve">precision = </t>
+  </si>
+  <si>
+    <t>TP / (TP + FN)</t>
+  </si>
+  <si>
+    <t>204/(204+44)=0.822</t>
+  </si>
+  <si>
+    <t>F - measure=</t>
+  </si>
+  <si>
+    <t>(2 * precision * recall) / (precision + recall)</t>
+  </si>
+  <si>
+    <t>(2*0.846*0.822)/(0.846+0.822) = 0.833</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
@@ -6842,7 +6888,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -6957,6 +7003,60 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color theme="8" tint="-0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="5" tint="-0.499984740745262"/>
+      </left>
+      <right style="thin">
+        <color theme="8" tint="-0.499984740745262"/>
+      </right>
+      <top style="thin">
+        <color theme="5" tint="-0.499984740745262"/>
+      </top>
+      <bottom style="thin">
+        <color theme="5" tint="-0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="8" tint="-0.499984740745262"/>
+      </left>
+      <right style="thin">
+        <color theme="5" tint="-0.499984740745262"/>
+      </right>
+      <top style="thin">
+        <color theme="5" tint="-0.499984740745262"/>
+      </top>
+      <bottom style="thin">
+        <color theme="8" tint="-0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="5" tint="-0.499984740745262"/>
+      </left>
+      <right style="thin">
+        <color theme="8" tint="-0.499984740745262"/>
+      </right>
+      <top style="thin">
+        <color theme="8" tint="-0.499984740745262"/>
+      </top>
+      <bottom style="thin">
+        <color theme="8" tint="-0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -7002,9 +7102,13 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -7359,7 +7463,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr filterMode="1"/>
   <dimension ref="A1:E2133"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -43629,7 +43733,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E2133">
+  <autoFilter ref="A1:E2133" xr:uid="{00000000-0009-0000-0000-000000000000}">
     <filterColumn colId="3">
       <filters>
         <filter val="TRUE"/>
@@ -43641,7 +43745,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:E248"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
@@ -47865,7 +47969,87 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E248"/>
+  <autoFilter ref="A1:E248" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02E6C42F-F785-AB44-9369-FA7EFFE3D8F0}">
+  <dimension ref="C2:G9"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="2" spans="3:7" x14ac:dyDescent="0.2">
+      <c r="D2" t="s">
+        <v>2159</v>
+      </c>
+      <c r="E2" t="s">
+        <v>2160</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>2161</v>
+      </c>
+    </row>
+    <row r="3" spans="3:7" x14ac:dyDescent="0.2">
+      <c r="C3" t="s">
+        <v>2162</v>
+      </c>
+      <c r="D3" s="3">
+        <v>44</v>
+      </c>
+      <c r="E3" s="4">
+        <v>204</v>
+      </c>
+      <c r="F3" s="5">
+        <v>37</v>
+      </c>
+      <c r="G3" t="s">
+        <v>2163</v>
+      </c>
+    </row>
+    <row r="7" spans="3:7" x14ac:dyDescent="0.2">
+      <c r="C7" t="s">
+        <v>2164</v>
+      </c>
+      <c r="D7" t="s">
+        <v>2165</v>
+      </c>
+      <c r="E7" t="s">
+        <v>2166</v>
+      </c>
+      <c r="F7" t="s">
+        <v>2167</v>
+      </c>
+    </row>
+    <row r="8" spans="3:7" x14ac:dyDescent="0.2">
+      <c r="C8" t="s">
+        <v>2168</v>
+      </c>
+      <c r="D8" t="s">
+        <v>2169</v>
+      </c>
+      <c r="E8" t="s">
+        <v>2166</v>
+      </c>
+      <c r="F8" t="s">
+        <v>2170</v>
+      </c>
+    </row>
+    <row r="9" spans="3:7" x14ac:dyDescent="0.2">
+      <c r="C9" t="s">
+        <v>2171</v>
+      </c>
+      <c r="D9" t="s">
+        <v>2172</v>
+      </c>
+      <c r="E9" t="s">
+        <v>2166</v>
+      </c>
+      <c r="F9" t="s">
+        <v>2173</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>